<commit_message>
Initial first dimension ddl (customer) and organaized in dwh folder
</commit_message>
<xml_diff>
--- a/docs/enterprise_data_warehouse_bus_matrix.xlsx
+++ b/docs/enterprise_data_warehouse_bus_matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahdi\Documents\GitHub\dwh-adventureworks\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5A302E6-5F05-4EF1-AEEE-E9E580B14F6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550C8BF0-5248-433C-958B-133AACE69AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="2" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1292" uniqueCount="478">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="490">
   <si>
     <t>Story Point Values</t>
   </si>
@@ -1516,6 +1516,42 @@
   </si>
   <si>
     <t>dim_store</t>
+  </si>
+  <si>
+    <t>store_key</t>
+  </si>
+  <si>
+    <t>store_name</t>
+  </si>
+  <si>
+    <t>square_feet</t>
+  </si>
+  <si>
+    <t>year_opened</t>
+  </si>
+  <si>
+    <t>number_employee</t>
+  </si>
+  <si>
+    <t>specialty</t>
+  </si>
+  <si>
+    <t>brands</t>
+  </si>
+  <si>
+    <t>Informationg about the store such as the square feet of store.</t>
+  </si>
+  <si>
+    <t>Informationg about the store such as number of employees.</t>
+  </si>
+  <si>
+    <t>Informationg about the store such as year oppend.</t>
+  </si>
+  <si>
+    <t>Informationg about the store such as speciality.</t>
+  </si>
+  <si>
+    <t>Number of brands available.</t>
   </si>
 </sst>
 </file>
@@ -2373,6 +2409,12 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" textRotation="90"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2415,18 +2457,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" textRotation="90"/>
-    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="25">
     <dxf>
       <font>
         <b/>
@@ -2435,6 +2471,13 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2716,12 +2759,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DimTypesTbl" displayName="DimTypesTbl" ref="A40:C50" totalsRowShown="0" dataDxfId="23">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DimTypesTbl" displayName="DimTypesTbl" ref="A40:C50" totalsRowShown="0" dataDxfId="24">
   <autoFilter ref="A40:C50" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Dimension Types" dataDxfId="22"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Definition" dataDxfId="21"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Ref" dataDxfId="20"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Dimension Types" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Definition" dataDxfId="22"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Ref" dataDxfId="21"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2732,7 +2775,7 @@
   <autoFilter ref="A84:C87" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Hub Types"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Definitions" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Definitions" dataDxfId="15"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Ref" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2752,8 +2795,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ObjectDefinition" displayName="ObjectDefinition" ref="A1:J107" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J107" xr:uid="{00000000-0009-0000-0100-000005000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ObjectDefinition" displayName="ObjectDefinition" ref="A1:J119" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:J119" xr:uid="{00000000-0009-0000-0100-000005000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -2782,12 +2825,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="FactTypesTbl" displayName="FactTypesTbl" ref="A30:C37" totalsRowShown="0" dataDxfId="19">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="FactTypesTbl" displayName="FactTypesTbl" ref="A30:C37" totalsRowShown="0" dataDxfId="20">
   <autoFilter ref="A30:C37" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Fact Types" dataDxfId="18"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Definition" dataDxfId="17"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Ref" dataDxfId="16"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Fact Types" dataDxfId="19"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Definition" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Ref" dataDxfId="17"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2838,7 +2881,7 @@
   <autoFilter ref="A53:C76" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Terms Dictionary"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Definition" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Definition" dataDxfId="16"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Ref"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4412,10 +4455,10 @@
       <c r="I8" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="J8" s="109" t="s">
+      <c r="J8" s="95" t="s">
         <v>236</v>
       </c>
-      <c r="K8" s="108" t="s">
+      <c r="K8" s="94" t="s">
         <v>237</v>
       </c>
       <c r="L8" s="89" t="s">
@@ -4682,13 +4725,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D12:D1048576 D3:D5 D7:D10">
-    <cfRule type="duplicateValues" dxfId="13" priority="131"/>
+    <cfRule type="duplicateValues" dxfId="14" priority="131"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL5:XFD5 B5:E5">
-    <cfRule type="duplicateValues" dxfId="12" priority="130"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="130"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5">
-    <cfRule type="duplicateValues" dxfId="11" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2">
     <cfRule type="colorScale" priority="121">
@@ -4727,10 +4770,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5">
-    <cfRule type="duplicateValues" dxfId="10" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5">
-    <cfRule type="duplicateValues" dxfId="9" priority="91"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9">
     <cfRule type="colorScale" priority="72">
@@ -4745,13 +4788,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE5 J5 O5">
-    <cfRule type="duplicateValues" dxfId="8" priority="457"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="457"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI5 X5">
-    <cfRule type="duplicateValues" dxfId="7" priority="475"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="475"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5">
-    <cfRule type="duplicateValues" dxfId="6" priority="852"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="852"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2">
     <cfRule type="colorScale" priority="853">
@@ -4766,7 +4809,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6">
-    <cfRule type="duplicateValues" dxfId="5" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6">
     <cfRule type="colorScale" priority="67">
@@ -4781,7 +4824,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ5 M5">
-    <cfRule type="duplicateValues" dxfId="4" priority="906"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="906"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2">
     <cfRule type="colorScale" priority="1082">
@@ -4808,7 +4851,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5">
-    <cfRule type="duplicateValues" dxfId="3" priority="1196"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="1196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:AJ2">
     <cfRule type="colorScale" priority="1426">
@@ -4835,7 +4878,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK5 N5 R5:W5 Y5:AD5 AF5:AH5 L5">
-    <cfRule type="duplicateValues" dxfId="2" priority="1430"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1430"/>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E9:E10 J6:AJ6" xr:uid="{00000000-0002-0000-0000-000002000000}">
@@ -4867,7 +4910,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J107"/>
+  <dimension ref="A1:J119"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -8029,18 +8072,308 @@
       <c r="C107" t="s">
         <v>477</v>
       </c>
+      <c r="D107" t="s">
+        <v>478</v>
+      </c>
+      <c r="E107" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A108" t="s">
+        <v>235</v>
+      </c>
+      <c r="B108" t="s">
+        <v>80</v>
+      </c>
+      <c r="C108" t="s">
+        <v>477</v>
+      </c>
+      <c r="D108" t="s">
+        <v>479</v>
+      </c>
+      <c r="E108" t="s">
+        <v>429</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A109" t="s">
+        <v>235</v>
+      </c>
+      <c r="B109" t="s">
+        <v>80</v>
+      </c>
+      <c r="C109" t="s">
+        <v>477</v>
+      </c>
+      <c r="D109" t="s">
+        <v>480</v>
+      </c>
+      <c r="E109" t="s">
+        <v>485</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A110" t="s">
+        <v>235</v>
+      </c>
+      <c r="B110" t="s">
+        <v>80</v>
+      </c>
+      <c r="C110" t="s">
+        <v>477</v>
+      </c>
+      <c r="D110" t="s">
+        <v>481</v>
+      </c>
+      <c r="E110" t="s">
+        <v>487</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A111" t="s">
+        <v>235</v>
+      </c>
+      <c r="B111" t="s">
+        <v>80</v>
+      </c>
+      <c r="C111" t="s">
+        <v>477</v>
+      </c>
+      <c r="D111" t="s">
+        <v>482</v>
+      </c>
+      <c r="E111" t="s">
+        <v>486</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A112" t="s">
+        <v>235</v>
+      </c>
+      <c r="B112" t="s">
+        <v>80</v>
+      </c>
+      <c r="C112" t="s">
+        <v>477</v>
+      </c>
+      <c r="D112" t="s">
+        <v>483</v>
+      </c>
+      <c r="E112" t="s">
+        <v>488</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A113" t="s">
+        <v>235</v>
+      </c>
+      <c r="B113" t="s">
+        <v>80</v>
+      </c>
+      <c r="C113" t="s">
+        <v>477</v>
+      </c>
+      <c r="D113" t="s">
+        <v>484</v>
+      </c>
+      <c r="E113" t="s">
+        <v>489</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A114" t="s">
+        <v>235</v>
+      </c>
+      <c r="B114" t="s">
+        <v>80</v>
+      </c>
+      <c r="C114" t="s">
+        <v>477</v>
+      </c>
+      <c r="D114" t="s">
+        <v>328</v>
+      </c>
+      <c r="E114" t="s">
+        <v>329</v>
+      </c>
+      <c r="F114" t="s">
+        <v>439</v>
+      </c>
+      <c r="G114" t="s">
+        <v>439</v>
+      </c>
+      <c r="H114" t="s">
+        <v>439</v>
+      </c>
+      <c r="I114" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A115" t="s">
+        <v>235</v>
+      </c>
+      <c r="B115" t="s">
+        <v>80</v>
+      </c>
+      <c r="C115" t="s">
+        <v>477</v>
+      </c>
+      <c r="D115" t="s">
+        <v>330</v>
+      </c>
+      <c r="E115" t="s">
+        <v>331</v>
+      </c>
+      <c r="F115" t="s">
+        <v>439</v>
+      </c>
+      <c r="G115" t="s">
+        <v>439</v>
+      </c>
+      <c r="H115" t="s">
+        <v>439</v>
+      </c>
+      <c r="I115" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A116" t="s">
+        <v>235</v>
+      </c>
+      <c r="B116" t="s">
+        <v>80</v>
+      </c>
+      <c r="C116" t="s">
+        <v>477</v>
+      </c>
+      <c r="D116" t="s">
+        <v>332</v>
+      </c>
+      <c r="E116" t="s">
+        <v>333</v>
+      </c>
+      <c r="F116" t="s">
+        <v>439</v>
+      </c>
+      <c r="G116" t="s">
+        <v>439</v>
+      </c>
+      <c r="H116" t="s">
+        <v>439</v>
+      </c>
+      <c r="I116" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A117" t="s">
+        <v>235</v>
+      </c>
+      <c r="B117" t="s">
+        <v>80</v>
+      </c>
+      <c r="C117" t="s">
+        <v>477</v>
+      </c>
+      <c r="D117" t="s">
+        <v>334</v>
+      </c>
+      <c r="E117" t="s">
+        <v>335</v>
+      </c>
+      <c r="F117" t="s">
+        <v>439</v>
+      </c>
+      <c r="G117" t="s">
+        <v>439</v>
+      </c>
+      <c r="H117" t="s">
+        <v>439</v>
+      </c>
+      <c r="I117" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A118" t="s">
+        <v>235</v>
+      </c>
+      <c r="B118" t="s">
+        <v>80</v>
+      </c>
+      <c r="C118" t="s">
+        <v>477</v>
+      </c>
+      <c r="D118" t="s">
+        <v>336</v>
+      </c>
+      <c r="E118" t="s">
+        <v>337</v>
+      </c>
+      <c r="F118" t="s">
+        <v>439</v>
+      </c>
+      <c r="G118" t="s">
+        <v>439</v>
+      </c>
+      <c r="H118" t="s">
+        <v>439</v>
+      </c>
+      <c r="I118" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A119" t="s">
+        <v>235</v>
+      </c>
+      <c r="B119" t="s">
+        <v>80</v>
+      </c>
+      <c r="C119" t="s">
+        <v>477</v>
+      </c>
+      <c r="D119" t="s">
+        <v>338</v>
+      </c>
+      <c r="E119" t="s">
+        <v>339</v>
+      </c>
+      <c r="F119" t="s">
+        <v>439</v>
+      </c>
+      <c r="G119" t="s">
+        <v>439</v>
+      </c>
+      <c r="H119" t="s">
+        <v>439</v>
+      </c>
+      <c r="I119" t="s">
+        <v>439</v>
+      </c>
+      <c r="J119" t="s">
+        <v>424</v>
+      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F109:F112">
-    <cfRule type="expression" dxfId="1" priority="1432">
+  <conditionalFormatting sqref="F113:F115">
+    <cfRule type="expression" dxfId="2" priority="1432">
+      <formula>AND($A112&lt;&gt;"", MOD(ROW(),2) = 0)</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F112">
+    <cfRule type="expression" dxfId="1" priority="1433">
       <formula>AND($A108&lt;&gt;"", MOD(ROW(),2) = 0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A107" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A119" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>SchemaList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B107" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B119" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>ObjectTypeList</formula1>
     </dataValidation>
   </dataValidations>
@@ -8088,54 +8421,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="94" t="s">
+      <c r="A1" s="96" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="105" t="s">
+      <c r="B1" s="107" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="98" t="s">
+      <c r="C1" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="99"/>
-      <c r="E1" s="98" t="s">
+      <c r="D1" s="101"/>
+      <c r="E1" s="100" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="100"/>
-      <c r="G1" s="101"/>
-      <c r="H1" s="102" t="s">
+      <c r="F1" s="102"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="103"/>
-      <c r="J1" s="104"/>
-      <c r="K1" s="102" t="s">
+      <c r="I1" s="105"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="104" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="104"/>
-      <c r="M1" s="102" t="s">
+      <c r="L1" s="106"/>
+      <c r="M1" s="104" t="s">
         <v>21</v>
       </c>
-      <c r="N1" s="96"/>
+      <c r="N1" s="98"/>
       <c r="O1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="102" t="s">
+      <c r="P1" s="104" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="104"/>
-      <c r="R1" s="98" t="s">
+      <c r="Q1" s="106"/>
+      <c r="R1" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="96" t="s">
+      <c r="S1" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="96" t="s">
+      <c r="T1" s="98" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="95"/>
-      <c r="B2" s="106"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="108"/>
       <c r="C2" s="11" t="s">
         <v>29</v>
       </c>
@@ -8181,9 +8514,9 @@
       <c r="Q2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="107"/>
-      <c r="S2" s="97"/>
-      <c r="T2" s="97"/>
+      <c r="R2" s="109"/>
+      <c r="S2" s="99"/>
+      <c r="T2" s="99"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>

</xml_diff>

<commit_message>
drop creation table's like customer, date, territory & store at dimension ddl.
</commit_message>
<xml_diff>
--- a/docs/enterprise_data_warehouse_bus_matrix.xlsx
+++ b/docs/enterprise_data_warehouse_bus_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahdi\Documents\GitHub\dwh-adventureworks\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{550C8BF0-5248-433C-958B-133AACE69AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C926F373-92B6-4741-B250-D45060625CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1379" uniqueCount="490">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="491">
   <si>
     <t>Story Point Values</t>
   </si>
@@ -1553,12 +1553,15 @@
   <si>
     <t>Number of brands available.</t>
   </si>
+  <si>
+    <t>Demographics</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1625,6 +1628,14 @@
       <name val="Consolas"/>
       <family val="3"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1" tint="4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="8">
     <fill>
@@ -1659,13 +1670,13 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFC000"/>
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2404,15 +2415,14 @@
     <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="7" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" textRotation="90"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2457,6 +2467,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -2466,11 +2477,21 @@
     <dxf>
       <font>
         <b/>
+        <strike val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1" tint="4.9989318521683403E-2"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
       </font>
       <fill>
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
-          <bgColor theme="7" tint="0.79998168889431442"/>
+          <bgColor theme="7"/>
         </patternFill>
       </fill>
     </dxf>
@@ -4455,10 +4476,10 @@
       <c r="I8" s="43" t="s">
         <v>46</v>
       </c>
-      <c r="J8" s="95" t="s">
+      <c r="J8" s="94" t="s">
         <v>236</v>
       </c>
-      <c r="K8" s="94" t="s">
+      <c r="K8" s="93" t="s">
         <v>237</v>
       </c>
       <c r="L8" s="89" t="s">
@@ -4926,34 +4947,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="109" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="91" t="s">
+      <c r="B1" s="109" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="91" t="s">
+      <c r="C1" s="109" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="91" t="s">
+      <c r="D1" s="109" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="91" t="s">
+      <c r="E1" s="109" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="91" t="s">
+      <c r="F1" s="109" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="91" t="s">
+      <c r="G1" s="109" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="91" t="s">
+      <c r="H1" s="109" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="91" t="s">
+      <c r="I1" s="109" t="s">
         <v>79</v>
       </c>
-      <c r="J1" s="91" t="s">
+      <c r="J1" s="109" t="s">
         <v>81</v>
       </c>
     </row>
@@ -8078,6 +8099,18 @@
       <c r="E107" t="s">
         <v>289</v>
       </c>
+      <c r="F107" t="s">
+        <v>439</v>
+      </c>
+      <c r="G107" t="s">
+        <v>439</v>
+      </c>
+      <c r="H107" t="s">
+        <v>439</v>
+      </c>
+      <c r="I107" t="s">
+        <v>439</v>
+      </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
@@ -8095,6 +8128,18 @@
       <c r="E108" t="s">
         <v>429</v>
       </c>
+      <c r="F108" t="s">
+        <v>393</v>
+      </c>
+      <c r="G108" t="s">
+        <v>394</v>
+      </c>
+      <c r="H108" t="s">
+        <v>402</v>
+      </c>
+      <c r="I108" t="s">
+        <v>430</v>
+      </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A109" t="s">
@@ -8112,6 +8157,18 @@
       <c r="E109" t="s">
         <v>485</v>
       </c>
+      <c r="F109" t="s">
+        <v>393</v>
+      </c>
+      <c r="G109" t="s">
+        <v>394</v>
+      </c>
+      <c r="H109" t="s">
+        <v>402</v>
+      </c>
+      <c r="I109" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A110" t="s">
@@ -8129,6 +8186,18 @@
       <c r="E110" t="s">
         <v>487</v>
       </c>
+      <c r="F110" t="s">
+        <v>393</v>
+      </c>
+      <c r="G110" t="s">
+        <v>394</v>
+      </c>
+      <c r="H110" t="s">
+        <v>402</v>
+      </c>
+      <c r="I110" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A111" t="s">
@@ -8146,6 +8215,18 @@
       <c r="E111" t="s">
         <v>486</v>
       </c>
+      <c r="F111" t="s">
+        <v>393</v>
+      </c>
+      <c r="G111" t="s">
+        <v>394</v>
+      </c>
+      <c r="H111" t="s">
+        <v>402</v>
+      </c>
+      <c r="I111" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A112" t="s">
@@ -8163,6 +8244,18 @@
       <c r="E112" t="s">
         <v>488</v>
       </c>
+      <c r="F112" t="s">
+        <v>393</v>
+      </c>
+      <c r="G112" t="s">
+        <v>394</v>
+      </c>
+      <c r="H112" t="s">
+        <v>402</v>
+      </c>
+      <c r="I112" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A113" t="s">
@@ -8180,6 +8273,18 @@
       <c r="E113" t="s">
         <v>489</v>
       </c>
+      <c r="F113" t="s">
+        <v>393</v>
+      </c>
+      <c r="G113" t="s">
+        <v>394</v>
+      </c>
+      <c r="H113" t="s">
+        <v>402</v>
+      </c>
+      <c r="I113" t="s">
+        <v>490</v>
+      </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A114" t="s">
@@ -8359,14 +8464,9 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="F113:F115">
+  <conditionalFormatting sqref="F114:F115">
     <cfRule type="expression" dxfId="2" priority="1432">
-      <formula>AND($A112&lt;&gt;"", MOD(ROW(),2) = 0)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F112">
-    <cfRule type="expression" dxfId="1" priority="1433">
-      <formula>AND($A108&lt;&gt;"", MOD(ROW(),2) = 0)</formula>
+      <formula>AND($A113&lt;&gt;"", MOD(ROW(),2) = 0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
@@ -8421,54 +8521,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="96" t="s">
+      <c r="A1" s="95" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="107" t="s">
+      <c r="B1" s="106" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="100" t="s">
+      <c r="C1" s="99" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="101"/>
-      <c r="E1" s="100" t="s">
+      <c r="D1" s="100"/>
+      <c r="E1" s="99" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="102"/>
-      <c r="G1" s="103"/>
-      <c r="H1" s="104" t="s">
+      <c r="F1" s="101"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="103" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="105"/>
-      <c r="J1" s="106"/>
-      <c r="K1" s="104" t="s">
+      <c r="I1" s="104"/>
+      <c r="J1" s="105"/>
+      <c r="K1" s="103" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="106"/>
-      <c r="M1" s="104" t="s">
+      <c r="L1" s="105"/>
+      <c r="M1" s="103" t="s">
         <v>21</v>
       </c>
-      <c r="N1" s="98"/>
+      <c r="N1" s="97"/>
       <c r="O1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="104" t="s">
+      <c r="P1" s="103" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="106"/>
-      <c r="R1" s="100" t="s">
+      <c r="Q1" s="105"/>
+      <c r="R1" s="99" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="98" t="s">
+      <c r="S1" s="97" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="98" t="s">
+      <c r="T1" s="97" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="97"/>
-      <c r="B2" s="108"/>
+      <c r="A2" s="96"/>
+      <c r="B2" s="107"/>
       <c r="C2" s="11" t="s">
         <v>29</v>
       </c>
@@ -8514,9 +8614,9 @@
       <c r="Q2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="109"/>
-      <c r="S2" s="99"/>
-      <c r="T2" s="99"/>
+      <c r="R2" s="108"/>
+      <c r="S2" s="98"/>
+      <c r="T2" s="98"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>
@@ -8621,15 +8721,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="92" t="s">
+      <c r="A1" s="91" t="s">
         <v>469</v>
       </c>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A2" s="92" t="s">
+      <c r="A2" s="91" t="s">
         <v>470</v>
       </c>
-      <c r="E2" s="93" t="str">
+      <c r="E2" s="92" t="str">
         <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(G2,FIND("]",G2)),"]",""),"[",""),"    ","")</f>
         <v>territory_key</v>
       </c>
@@ -8654,7 +8754,7 @@
       <c r="D3" s="83" t="s">
         <v>445</v>
       </c>
-      <c r="E3" s="93" t="str">
+      <c r="E3" s="92" t="str">
         <f t="shared" ref="E3:E6" si="0">SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(G3,FIND("]",G3)),"]",""),"[",""),"    ","")</f>
         <v>territory_name_bk</v>
       </c>
@@ -8679,7 +8779,7 @@
       <c r="D4" s="83" t="s">
         <v>433</v>
       </c>
-      <c r="E4" s="93" t="str">
+      <c r="E4" s="92" t="str">
         <f t="shared" si="0"/>
         <v>territory_group</v>
       </c>
@@ -8704,7 +8804,7 @@
       <c r="D5" s="83" t="s">
         <v>434</v>
       </c>
-      <c r="E5" s="93" t="str">
+      <c r="E5" s="92" t="str">
         <f t="shared" si="0"/>
         <v>country_region_code</v>
       </c>
@@ -8729,7 +8829,7 @@
       <c r="D6" s="83" t="s">
         <v>435</v>
       </c>
-      <c r="E6" s="93" t="str">
+      <c r="E6" s="92" t="str">
         <f t="shared" si="0"/>
         <v>country_name</v>
       </c>

</xml_diff>

<commit_message>
Updates: 1- Checking data quality in Store and Employee 2- Change data type and initial transform ddl for employee and person table 3- initial dimenson of salesperson on یصا 4- insert some necessary columns in extract tables layer 5- create and test ssis solution form store and salesperson. changing some flow to fit archetecture 6- setup dim_salesperson busmatrix inputs
</commit_message>
<xml_diff>
--- a/docs/enterprise_data_warehouse_bus_matrix.xlsx
+++ b/docs/enterprise_data_warehouse_bus_matrix.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahdi\Documents\GitHub\dwh-adventureworks\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C926F373-92B6-4741-B250-D45060625CE6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794E7F44-0641-4FE3-920A-BD61679924D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1407" uniqueCount="491">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1468" uniqueCount="498">
   <si>
     <t>Story Point Values</t>
   </si>
@@ -1555,6 +1555,27 @@
   </si>
   <si>
     <t>Demographics</t>
+  </si>
+  <si>
+    <t>dim_salesperson</t>
+  </si>
+  <si>
+    <t>salesperson_key</t>
+  </si>
+  <si>
+    <t>national_number_bk</t>
+  </si>
+  <si>
+    <t>full_name</t>
+  </si>
+  <si>
+    <t>job_title</t>
+  </si>
+  <si>
+    <t>hire_date</t>
+  </si>
+  <si>
+    <t>is_current_employee</t>
   </si>
 </sst>
 </file>
@@ -2425,6 +2446,7 @@
     <xf numFmtId="0" fontId="6" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" textRotation="90"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2467,13 +2489,12 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="25">
+  <dxfs count="24">
     <dxf>
       <font>
         <b/>
@@ -2492,13 +2513,6 @@
         <patternFill patternType="solid">
           <fgColor indexed="64"/>
           <bgColor theme="7"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
         </patternFill>
       </fill>
     </dxf>
@@ -2780,12 +2794,12 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DimTypesTbl" displayName="DimTypesTbl" ref="A40:C50" totalsRowShown="0" dataDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF01000000}" name="DimTypesTbl" displayName="DimTypesTbl" ref="A40:C50" totalsRowShown="0" dataDxfId="23">
   <autoFilter ref="A40:C50" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Dimension Types" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Definition" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Ref" dataDxfId="21"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0100-000001000000}" name="Dimension Types" dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0100-000002000000}" name="Definition" dataDxfId="21"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0100-000003000000}" name="Ref" dataDxfId="20"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2796,7 +2810,7 @@
   <autoFilter ref="A84:C87" xr:uid="{00000000-0009-0000-0100-00000B000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0A00-000001000000}" name="Hub Types"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Definitions" dataDxfId="15"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0A00-000002000000}" name="Definitions" dataDxfId="14"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0A00-000003000000}" name="Ref" dataCellStyle="Hyperlink"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -2816,8 +2830,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ObjectDefinition" displayName="ObjectDefinition" ref="A1:J119" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:J119" xr:uid="{00000000-0009-0000-0100-000005000000}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="ObjectDefinition" displayName="ObjectDefinition" ref="A1:J131" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:J131" xr:uid="{00000000-0009-0000-0100-000005000000}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -2846,12 +2860,12 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="FactTypesTbl" displayName="FactTypesTbl" ref="A30:C37" totalsRowShown="0" dataDxfId="20">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{00000000-000C-0000-FFFF-FFFF02000000}" name="FactTypesTbl" displayName="FactTypesTbl" ref="A30:C37" totalsRowShown="0" dataDxfId="19">
   <autoFilter ref="A30:C37" xr:uid="{00000000-0009-0000-0100-000002000000}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Fact Types" dataDxfId="19"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Definition" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Ref" dataDxfId="17"/>
+    <tableColumn id="1" xr3:uid="{00000000-0010-0000-0200-000001000000}" name="Fact Types" dataDxfId="18"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0200-000002000000}" name="Definition" dataDxfId="17"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0200-000003000000}" name="Ref" dataDxfId="16"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2902,7 +2916,7 @@
   <autoFilter ref="A53:C76" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="3">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0700-000001000000}" name="Terms Dictionary"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Definition" dataDxfId="16"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0700-000002000000}" name="Definition" dataDxfId="15"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0700-000003000000}" name="Ref"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -4746,13 +4760,13 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D12:D1048576 D3:D5 D7:D10">
-    <cfRule type="duplicateValues" dxfId="14" priority="131"/>
+    <cfRule type="duplicateValues" dxfId="13" priority="131"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AL5:XFD5 B5:E5">
-    <cfRule type="duplicateValues" dxfId="13" priority="130"/>
+    <cfRule type="duplicateValues" dxfId="12" priority="130"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5">
-    <cfRule type="duplicateValues" dxfId="12" priority="122"/>
+    <cfRule type="duplicateValues" dxfId="11" priority="122"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2">
     <cfRule type="colorScale" priority="121">
@@ -4791,10 +4805,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="Q5">
-    <cfRule type="duplicateValues" dxfId="11" priority="97"/>
+    <cfRule type="duplicateValues" dxfId="10" priority="97"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="P5">
-    <cfRule type="duplicateValues" dxfId="10" priority="91"/>
+    <cfRule type="duplicateValues" dxfId="9" priority="91"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A9">
     <cfRule type="colorScale" priority="72">
@@ -4809,13 +4823,13 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AE5 J5 O5">
-    <cfRule type="duplicateValues" dxfId="9" priority="457"/>
+    <cfRule type="duplicateValues" dxfId="8" priority="457"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="AI5 X5">
-    <cfRule type="duplicateValues" dxfId="8" priority="475"/>
+    <cfRule type="duplicateValues" dxfId="7" priority="475"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I5">
-    <cfRule type="duplicateValues" dxfId="7" priority="852"/>
+    <cfRule type="duplicateValues" dxfId="6" priority="852"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="I2">
     <cfRule type="colorScale" priority="853">
@@ -4830,7 +4844,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="D6">
-    <cfRule type="duplicateValues" dxfId="6" priority="68"/>
+    <cfRule type="duplicateValues" dxfId="5" priority="68"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="A6">
     <cfRule type="colorScale" priority="67">
@@ -4845,7 +4859,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AJ5 M5">
-    <cfRule type="duplicateValues" dxfId="5" priority="906"/>
+    <cfRule type="duplicateValues" dxfId="4" priority="906"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="J2">
     <cfRule type="colorScale" priority="1082">
@@ -4872,7 +4886,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K5">
-    <cfRule type="duplicateValues" dxfId="4" priority="1196"/>
+    <cfRule type="duplicateValues" dxfId="3" priority="1196"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="K2:AJ2">
     <cfRule type="colorScale" priority="1426">
@@ -4899,7 +4913,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="AK5 N5 R5:W5 Y5:AD5 AF5:AH5 L5">
-    <cfRule type="duplicateValues" dxfId="3" priority="1430"/>
+    <cfRule type="duplicateValues" dxfId="2" priority="1430"/>
   </conditionalFormatting>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="E9:E10 J6:AJ6" xr:uid="{00000000-0002-0000-0000-000002000000}">
@@ -4931,7 +4945,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
-  <dimension ref="A1:J119"/>
+  <dimension ref="A1:J131"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
@@ -4947,34 +4961,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A1" s="109" t="s">
+      <c r="A1" s="95" t="s">
         <v>72</v>
       </c>
-      <c r="B1" s="109" t="s">
+      <c r="B1" s="95" t="s">
         <v>73</v>
       </c>
-      <c r="C1" s="109" t="s">
+      <c r="C1" s="95" t="s">
         <v>74</v>
       </c>
-      <c r="D1" s="109" t="s">
+      <c r="D1" s="95" t="s">
         <v>75</v>
       </c>
-      <c r="E1" s="109" t="s">
+      <c r="E1" s="95" t="s">
         <v>83</v>
       </c>
-      <c r="F1" s="109" t="s">
+      <c r="F1" s="95" t="s">
         <v>76</v>
       </c>
-      <c r="G1" s="109" t="s">
+      <c r="G1" s="95" t="s">
         <v>77</v>
       </c>
-      <c r="H1" s="109" t="s">
+      <c r="H1" s="95" t="s">
         <v>78</v>
       </c>
-      <c r="I1" s="109" t="s">
+      <c r="I1" s="95" t="s">
         <v>79</v>
       </c>
-      <c r="J1" s="109" t="s">
+      <c r="J1" s="95" t="s">
         <v>81</v>
       </c>
     </row>
@@ -8463,17 +8477,224 @@
         <v>424</v>
       </c>
     </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A120" t="s">
+        <v>235</v>
+      </c>
+      <c r="B120" t="s">
+        <v>80</v>
+      </c>
+      <c r="C120" t="s">
+        <v>491</v>
+      </c>
+      <c r="D120" t="s">
+        <v>492</v>
+      </c>
+      <c r="E120" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A121" t="s">
+        <v>235</v>
+      </c>
+      <c r="B121" t="s">
+        <v>80</v>
+      </c>
+      <c r="C121" t="s">
+        <v>491</v>
+      </c>
+      <c r="D121" t="s">
+        <v>493</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A122" t="s">
+        <v>235</v>
+      </c>
+      <c r="B122" t="s">
+        <v>80</v>
+      </c>
+      <c r="C122" t="s">
+        <v>491</v>
+      </c>
+      <c r="D122" t="s">
+        <v>494</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A123" t="s">
+        <v>235</v>
+      </c>
+      <c r="B123" t="s">
+        <v>80</v>
+      </c>
+      <c r="C123" t="s">
+        <v>491</v>
+      </c>
+      <c r="D123" t="s">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A124" t="s">
+        <v>235</v>
+      </c>
+      <c r="B124" t="s">
+        <v>80</v>
+      </c>
+      <c r="C124" t="s">
+        <v>491</v>
+      </c>
+      <c r="D124" t="s">
+        <v>496</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A125" t="s">
+        <v>235</v>
+      </c>
+      <c r="B125" t="s">
+        <v>80</v>
+      </c>
+      <c r="C125" t="s">
+        <v>491</v>
+      </c>
+      <c r="D125" t="s">
+        <v>497</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A126" t="s">
+        <v>235</v>
+      </c>
+      <c r="B126" t="s">
+        <v>80</v>
+      </c>
+      <c r="C126" t="s">
+        <v>491</v>
+      </c>
+      <c r="D126" t="s">
+        <v>328</v>
+      </c>
+      <c r="E126" t="s">
+        <v>329</v>
+      </c>
+      <c r="F126" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A127" t="s">
+        <v>235</v>
+      </c>
+      <c r="B127" t="s">
+        <v>80</v>
+      </c>
+      <c r="C127" t="s">
+        <v>491</v>
+      </c>
+      <c r="D127" t="s">
+        <v>330</v>
+      </c>
+      <c r="E127" t="s">
+        <v>331</v>
+      </c>
+      <c r="F127" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A128" t="s">
+        <v>235</v>
+      </c>
+      <c r="B128" t="s">
+        <v>80</v>
+      </c>
+      <c r="C128" t="s">
+        <v>491</v>
+      </c>
+      <c r="D128" t="s">
+        <v>332</v>
+      </c>
+      <c r="E128" t="s">
+        <v>333</v>
+      </c>
+      <c r="F128" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A129" t="s">
+        <v>235</v>
+      </c>
+      <c r="B129" t="s">
+        <v>80</v>
+      </c>
+      <c r="C129" t="s">
+        <v>491</v>
+      </c>
+      <c r="D129" t="s">
+        <v>334</v>
+      </c>
+      <c r="E129" t="s">
+        <v>335</v>
+      </c>
+      <c r="F129" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A130" t="s">
+        <v>235</v>
+      </c>
+      <c r="B130" t="s">
+        <v>80</v>
+      </c>
+      <c r="C130" t="s">
+        <v>491</v>
+      </c>
+      <c r="D130" t="s">
+        <v>336</v>
+      </c>
+      <c r="E130" t="s">
+        <v>337</v>
+      </c>
+      <c r="F130" t="s">
+        <v>439</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A131" t="s">
+        <v>235</v>
+      </c>
+      <c r="B131" t="s">
+        <v>80</v>
+      </c>
+      <c r="C131" t="s">
+        <v>491</v>
+      </c>
+      <c r="D131" t="s">
+        <v>338</v>
+      </c>
+      <c r="E131" t="s">
+        <v>339</v>
+      </c>
+      <c r="F131" t="s">
+        <v>439</v>
+      </c>
+    </row>
   </sheetData>
   <conditionalFormatting sqref="F114:F115">
-    <cfRule type="expression" dxfId="2" priority="1432">
+    <cfRule type="expression" dxfId="1" priority="1432">
       <formula>AND($A113&lt;&gt;"", MOD(ROW(),2) = 0)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A119" xr:uid="{00000000-0002-0000-0100-000000000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="A2:A131" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>SchemaList</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B119" xr:uid="{00000000-0002-0000-0100-000001000000}">
+    <dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="B2:B131" xr:uid="{00000000-0002-0000-0100-000001000000}">
       <formula1>ObjectTypeList</formula1>
     </dataValidation>
   </dataValidations>
@@ -8521,54 +8742,54 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.25">
-      <c r="A1" s="95" t="s">
+      <c r="A1" s="96" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="106" t="s">
+      <c r="B1" s="107" t="s">
         <v>28</v>
       </c>
-      <c r="C1" s="99" t="s">
+      <c r="C1" s="100" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="100"/>
-      <c r="E1" s="99" t="s">
+      <c r="D1" s="101"/>
+      <c r="E1" s="100" t="s">
         <v>12</v>
       </c>
-      <c r="F1" s="101"/>
-      <c r="G1" s="102"/>
-      <c r="H1" s="103" t="s">
+      <c r="F1" s="102"/>
+      <c r="G1" s="103"/>
+      <c r="H1" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="I1" s="104"/>
-      <c r="J1" s="105"/>
-      <c r="K1" s="103" t="s">
+      <c r="I1" s="105"/>
+      <c r="J1" s="106"/>
+      <c r="K1" s="104" t="s">
         <v>18</v>
       </c>
-      <c r="L1" s="105"/>
-      <c r="M1" s="103" t="s">
+      <c r="L1" s="106"/>
+      <c r="M1" s="104" t="s">
         <v>21</v>
       </c>
-      <c r="N1" s="97"/>
+      <c r="N1" s="98"/>
       <c r="O1" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="P1" s="103" t="s">
+      <c r="P1" s="104" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="105"/>
-      <c r="R1" s="99" t="s">
+      <c r="Q1" s="106"/>
+      <c r="R1" s="100" t="s">
         <v>32</v>
       </c>
-      <c r="S1" s="97" t="s">
+      <c r="S1" s="98" t="s">
         <v>33</v>
       </c>
-      <c r="T1" s="97" t="s">
+      <c r="T1" s="98" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="2" spans="1:20" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="96"/>
-      <c r="B2" s="107"/>
+      <c r="A2" s="97"/>
+      <c r="B2" s="108"/>
       <c r="C2" s="11" t="s">
         <v>29</v>
       </c>
@@ -8614,9 +8835,9 @@
       <c r="Q2" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="R2" s="108"/>
-      <c r="S2" s="98"/>
-      <c r="T2" s="98"/>
+      <c r="R2" s="109"/>
+      <c r="S2" s="99"/>
+      <c r="T2" s="99"/>
     </row>
     <row r="3" spans="1:20" x14ac:dyDescent="0.25">
       <c r="A3" s="15"/>

</xml_diff>

<commit_message>
1- Changes OLTP source in busmatrix excel. 2- Update Datatype's in Extract table. 3- Check Datatype in Salesorderdetails.
</commit_message>
<xml_diff>
--- a/docs/enterprise_data_warehouse_bus_matrix.xlsx
+++ b/docs/enterprise_data_warehouse_bus_matrix.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Mahdi\Documents\GitHub\dwh-adventureworks\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B1DB6C9-67D3-44A1-8CA6-ED2252BCC022}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D01E15A-DFBC-4E75-BA9A-9901F1356641}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="16440" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Definitions" sheetId="2" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1665" uniqueCount="533">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1631" uniqueCount="506">
   <si>
     <t>Story Point Values</t>
   </si>
@@ -1416,87 +1416,6 @@
     <t>Data warehouse Primary Key.</t>
   </si>
   <si>
-    <t>Primary key for SalesTerritory records.</t>
-  </si>
-  <si>
-    <t>SalesYTD</t>
-  </si>
-  <si>
-    <t>Sales in the territory year to date.</t>
-  </si>
-  <si>
-    <t>SalesLastYear</t>
-  </si>
-  <si>
-    <t>Sales in the territory the previous year.</t>
-  </si>
-  <si>
-    <t>CostYTD</t>
-  </si>
-  <si>
-    <t>Business costs in the territory year to date.</t>
-  </si>
-  <si>
-    <t>CostLastYear</t>
-  </si>
-  <si>
-    <t>Business costs in the territory the previous year.</t>
-  </si>
-  <si>
-    <t>rowguid</t>
-  </si>
-  <si>
-    <t>ROWGUIDCOL number uniquely identifying the record. Used to support a merge replication sample.</t>
-  </si>
-  <si>
-    <t>ModifiedDate</t>
-  </si>
-  <si>
-    <t>Date and time the record was last updated.</t>
-  </si>
-  <si>
-    <t>-- System metadata attributes.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">    [sys_source_record_id] </t>
-  </si>
-  <si>
-    <t>    [territory_name_bk]         NVARCHAR (20)       NOT NULL,   --</t>
-  </si>
-  <si>
-    <t>    [territory_group]           NVARCHAR (20)       NOT NULL,</t>
-  </si>
-  <si>
-    <t>    [country_region_code]       NVARCHAR (5)        NOT NULL,</t>
-  </si>
-  <si>
-    <t>    [country_name]              NVARCHAR (30)       NOT NULL,</t>
-  </si>
-  <si>
-    <t>    [sys_insert_date]         DATETIME2(3)        NOT NULL,   -- System metadata: date and time when the record was inserted.</t>
-  </si>
-  <si>
-    <t>    [sys_update_date]         DATETIME2(3)            NULL,   -- System metadata: date and time when the record was last updated.</t>
-  </si>
-  <si>
-    <t>    [sys_delete_date]         DATETIME2(3)            NULL,   -- System metadata: date and time when the record was deleted or marked for deletion.</t>
-  </si>
-  <si>
-    <t>    [sys_hash_value]          CHAR(64)            NOT NULL,   -- System metadata: hash value used to detect changes in source attributes.</t>
-  </si>
-  <si>
-    <t>    [sys_data_source]         NVARCHAR(25)        NOT NULL,   -- System metadata: name of the source system.</t>
-  </si>
-  <si>
-    <t>=LEFT(A1,FIND(" ",A1)-1)</t>
-  </si>
-  <si>
-    <t>=MID(A1,FIND("-- ",A1)+3,LEN(A1))</t>
-  </si>
-  <si>
-    <t>[territory_key]             INT IDENTITY (1, 1) NOT NULL,   -- Surrogate key generated by the data warehouse.</t>
-  </si>
-  <si>
     <t>territory_name_bk</t>
   </si>
   <si>
@@ -1578,9 +1497,6 @@
     <t>AdventureWorks2024</t>
   </si>
   <si>
-    <t>Each row per product sold.</t>
-  </si>
-  <si>
     <t>Concatenate first name &amp; last name of source system.</t>
   </si>
   <si>
@@ -1599,9 +1515,6 @@
     <t>SalesOrderDetailID</t>
   </si>
   <si>
-    <t>sales_order_id_bk</t>
-  </si>
-  <si>
     <t>SalesOrderID</t>
   </si>
   <si>
@@ -1681,6 +1594,12 @@
   </si>
   <si>
     <t>Bring with lookup</t>
+  </si>
+  <si>
+    <t>sales_order_id</t>
+  </si>
+  <si>
+    <t>One row per sales order line item</t>
   </si>
 </sst>
 </file>
@@ -4601,10 +4520,10 @@
         <v>387</v>
       </c>
       <c r="N8" s="89" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="O8" s="108" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="P8" s="44"/>
       <c r="Q8" s="44"/>
@@ -4653,7 +4572,7 @@
         <v>50</v>
       </c>
       <c r="I9" s="52" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="J9" s="53" t="s">
         <v>5</v>
@@ -4759,10 +4678,10 @@
         <v>387</v>
       </c>
       <c r="N11" s="68" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="O11" s="69" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="P11" s="67"/>
       <c r="Q11" s="67"/>
@@ -5125,7 +5044,7 @@
         <v>438</v>
       </c>
       <c r="J2" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
@@ -5157,7 +5076,7 @@
         <v>438</v>
       </c>
       <c r="J3" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
@@ -5189,7 +5108,7 @@
         <v>438</v>
       </c>
       <c r="J4" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
@@ -5221,7 +5140,7 @@
         <v>438</v>
       </c>
       <c r="J5" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -5253,7 +5172,7 @@
         <v>438</v>
       </c>
       <c r="J6" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
@@ -5285,7 +5204,7 @@
         <v>438</v>
       </c>
       <c r="J7" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
@@ -5317,7 +5236,7 @@
         <v>438</v>
       </c>
       <c r="J8" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
@@ -5349,7 +5268,7 @@
         <v>438</v>
       </c>
       <c r="J9" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
@@ -5381,7 +5300,7 @@
         <v>438</v>
       </c>
       <c r="J10" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
@@ -5413,7 +5332,7 @@
         <v>438</v>
       </c>
       <c r="J11" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.25">
@@ -5445,7 +5364,7 @@
         <v>438</v>
       </c>
       <c r="J12" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="13" spans="1:10" x14ac:dyDescent="0.25">
@@ -5477,7 +5396,7 @@
         <v>438</v>
       </c>
       <c r="J13" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.25">
@@ -5509,7 +5428,7 @@
         <v>438</v>
       </c>
       <c r="J14" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.25">
@@ -5541,7 +5460,7 @@
         <v>438</v>
       </c>
       <c r="J15" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.25">
@@ -5573,7 +5492,7 @@
         <v>438</v>
       </c>
       <c r="J16" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.25">
@@ -5605,7 +5524,7 @@
         <v>438</v>
       </c>
       <c r="J17" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.25">
@@ -5637,7 +5556,7 @@
         <v>438</v>
       </c>
       <c r="J18" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.25">
@@ -5669,7 +5588,7 @@
         <v>438</v>
       </c>
       <c r="J19" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.25">
@@ -5701,7 +5620,7 @@
         <v>438</v>
       </c>
       <c r="J20" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.25">
@@ -5733,7 +5652,7 @@
         <v>438</v>
       </c>
       <c r="J21" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.25">
@@ -5765,7 +5684,7 @@
         <v>438</v>
       </c>
       <c r="J22" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.25">
@@ -5797,7 +5716,7 @@
         <v>438</v>
       </c>
       <c r="J23" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="24" spans="1:10" x14ac:dyDescent="0.25">
@@ -5829,7 +5748,7 @@
         <v>438</v>
       </c>
       <c r="J24" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="25" spans="1:10" x14ac:dyDescent="0.25">
@@ -5861,7 +5780,7 @@
         <v>438</v>
       </c>
       <c r="J25" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="26" spans="1:10" x14ac:dyDescent="0.25">
@@ -5893,7 +5812,7 @@
         <v>438</v>
       </c>
       <c r="J26" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="27" spans="1:10" x14ac:dyDescent="0.25">
@@ -5925,7 +5844,7 @@
         <v>438</v>
       </c>
       <c r="J27" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="28" spans="1:10" x14ac:dyDescent="0.25">
@@ -5957,7 +5876,7 @@
         <v>438</v>
       </c>
       <c r="J28" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="29" spans="1:10" x14ac:dyDescent="0.25">
@@ -5989,7 +5908,7 @@
         <v>438</v>
       </c>
       <c r="J29" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="30" spans="1:10" x14ac:dyDescent="0.25">
@@ -6021,7 +5940,7 @@
         <v>438</v>
       </c>
       <c r="J30" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="31" spans="1:10" x14ac:dyDescent="0.25">
@@ -6053,7 +5972,7 @@
         <v>438</v>
       </c>
       <c r="J31" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="32" spans="1:10" x14ac:dyDescent="0.25">
@@ -6085,7 +6004,7 @@
         <v>438</v>
       </c>
       <c r="J32" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="33" spans="1:10" x14ac:dyDescent="0.25">
@@ -6117,7 +6036,7 @@
         <v>438</v>
       </c>
       <c r="J33" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="34" spans="1:10" x14ac:dyDescent="0.25">
@@ -6149,7 +6068,7 @@
         <v>438</v>
       </c>
       <c r="J34" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="35" spans="1:10" x14ac:dyDescent="0.25">
@@ -6181,7 +6100,7 @@
         <v>438</v>
       </c>
       <c r="J35" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="36" spans="1:10" x14ac:dyDescent="0.25">
@@ -6213,7 +6132,7 @@
         <v>438</v>
       </c>
       <c r="J36" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="37" spans="1:10" x14ac:dyDescent="0.25">
@@ -6245,7 +6164,7 @@
         <v>438</v>
       </c>
       <c r="J37" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="38" spans="1:10" x14ac:dyDescent="0.25">
@@ -6277,7 +6196,7 @@
         <v>438</v>
       </c>
       <c r="J38" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="39" spans="1:10" x14ac:dyDescent="0.25">
@@ -6309,7 +6228,7 @@
         <v>438</v>
       </c>
       <c r="J39" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="40" spans="1:10" x14ac:dyDescent="0.25">
@@ -6341,7 +6260,7 @@
         <v>438</v>
       </c>
       <c r="J40" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="41" spans="1:10" x14ac:dyDescent="0.25">
@@ -6373,7 +6292,7 @@
         <v>438</v>
       </c>
       <c r="J41" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="42" spans="1:10" x14ac:dyDescent="0.25">
@@ -6405,7 +6324,7 @@
         <v>438</v>
       </c>
       <c r="J42" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="43" spans="1:10" x14ac:dyDescent="0.25">
@@ -6437,7 +6356,7 @@
         <v>438</v>
       </c>
       <c r="J43" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="44" spans="1:10" x14ac:dyDescent="0.25">
@@ -6469,7 +6388,7 @@
         <v>438</v>
       </c>
       <c r="J44" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="45" spans="1:10" x14ac:dyDescent="0.25">
@@ -6501,7 +6420,7 @@
         <v>438</v>
       </c>
       <c r="J45" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="46" spans="1:10" x14ac:dyDescent="0.25">
@@ -6533,7 +6452,7 @@
         <v>438</v>
       </c>
       <c r="J46" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="47" spans="1:10" x14ac:dyDescent="0.25">
@@ -6565,7 +6484,7 @@
         <v>438</v>
       </c>
       <c r="J47" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="48" spans="1:10" x14ac:dyDescent="0.25">
@@ -6597,7 +6516,7 @@
         <v>438</v>
       </c>
       <c r="J48" t="s">
-        <v>502</v>
+        <v>474</v>
       </c>
     </row>
     <row r="49" spans="1:10" x14ac:dyDescent="0.25">
@@ -7919,7 +7838,7 @@
         <v>387</v>
       </c>
       <c r="D97" s="28" t="s">
-        <v>471</v>
+        <v>444</v>
       </c>
       <c r="E97" t="s">
         <v>432</v>
@@ -8006,10 +7925,10 @@
         <v>387</v>
       </c>
       <c r="D100" s="28" t="s">
-        <v>472</v>
+        <v>445</v>
       </c>
       <c r="E100" t="s">
-        <v>473</v>
+        <v>446</v>
       </c>
       <c r="F100" t="s">
         <v>392</v>
@@ -8018,7 +7937,7 @@
         <v>400</v>
       </c>
       <c r="H100" t="s">
-        <v>474</v>
+        <v>447</v>
       </c>
       <c r="I100" t="s">
         <v>429</v>
@@ -8209,10 +8128,10 @@
         <v>80</v>
       </c>
       <c r="C107" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D107" t="s">
-        <v>476</v>
+        <v>449</v>
       </c>
       <c r="E107" t="s">
         <v>288</v>
@@ -8238,10 +8157,10 @@
         <v>80</v>
       </c>
       <c r="C108" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D108" t="s">
-        <v>477</v>
+        <v>450</v>
       </c>
       <c r="E108" t="s">
         <v>428</v>
@@ -8267,13 +8186,13 @@
         <v>80</v>
       </c>
       <c r="C109" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D109" t="s">
-        <v>478</v>
+        <v>451</v>
       </c>
       <c r="E109" t="s">
-        <v>483</v>
+        <v>456</v>
       </c>
       <c r="F109" t="s">
         <v>392</v>
@@ -8285,7 +8204,7 @@
         <v>401</v>
       </c>
       <c r="I109" t="s">
-        <v>488</v>
+        <v>461</v>
       </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.25">
@@ -8296,13 +8215,13 @@
         <v>80</v>
       </c>
       <c r="C110" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D110" t="s">
-        <v>479</v>
+        <v>452</v>
       </c>
       <c r="E110" t="s">
-        <v>485</v>
+        <v>458</v>
       </c>
       <c r="F110" t="s">
         <v>392</v>
@@ -8314,7 +8233,7 @@
         <v>401</v>
       </c>
       <c r="I110" t="s">
-        <v>488</v>
+        <v>461</v>
       </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.25">
@@ -8325,13 +8244,13 @@
         <v>80</v>
       </c>
       <c r="C111" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D111" t="s">
-        <v>480</v>
+        <v>453</v>
       </c>
       <c r="E111" t="s">
-        <v>484</v>
+        <v>457</v>
       </c>
       <c r="F111" t="s">
         <v>392</v>
@@ -8343,7 +8262,7 @@
         <v>401</v>
       </c>
       <c r="I111" t="s">
-        <v>488</v>
+        <v>461</v>
       </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.25">
@@ -8354,13 +8273,13 @@
         <v>80</v>
       </c>
       <c r="C112" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D112" t="s">
-        <v>481</v>
+        <v>454</v>
       </c>
       <c r="E112" t="s">
-        <v>486</v>
+        <v>459</v>
       </c>
       <c r="F112" t="s">
         <v>392</v>
@@ -8372,7 +8291,7 @@
         <v>401</v>
       </c>
       <c r="I112" t="s">
-        <v>488</v>
+        <v>461</v>
       </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.25">
@@ -8383,13 +8302,13 @@
         <v>80</v>
       </c>
       <c r="C113" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D113" t="s">
-        <v>482</v>
+        <v>455</v>
       </c>
       <c r="E113" t="s">
-        <v>487</v>
+        <v>460</v>
       </c>
       <c r="F113" t="s">
         <v>392</v>
@@ -8401,7 +8320,7 @@
         <v>401</v>
       </c>
       <c r="I113" t="s">
-        <v>488</v>
+        <v>461</v>
       </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.25">
@@ -8412,7 +8331,7 @@
         <v>80</v>
       </c>
       <c r="C114" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D114" t="s">
         <v>327</v>
@@ -8441,7 +8360,7 @@
         <v>80</v>
       </c>
       <c r="C115" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D115" t="s">
         <v>329</v>
@@ -8470,7 +8389,7 @@
         <v>80</v>
       </c>
       <c r="C116" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D116" t="s">
         <v>331</v>
@@ -8499,7 +8418,7 @@
         <v>80</v>
       </c>
       <c r="C117" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D117" t="s">
         <v>333</v>
@@ -8528,7 +8447,7 @@
         <v>80</v>
       </c>
       <c r="C118" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D118" t="s">
         <v>335</v>
@@ -8557,7 +8476,7 @@
         <v>80</v>
       </c>
       <c r="C119" t="s">
-        <v>475</v>
+        <v>448</v>
       </c>
       <c r="D119" t="s">
         <v>337</v>
@@ -8589,10 +8508,10 @@
         <v>80</v>
       </c>
       <c r="C120" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D120" t="s">
-        <v>490</v>
+        <v>463</v>
       </c>
       <c r="E120" t="s">
         <v>288</v>
@@ -8609,10 +8528,10 @@
         <v>80</v>
       </c>
       <c r="C121" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D121" t="s">
-        <v>491</v>
+        <v>464</v>
       </c>
       <c r="F121" t="s">
         <v>392</v>
@@ -8626,13 +8545,13 @@
         <v>80</v>
       </c>
       <c r="C122" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D122" t="s">
-        <v>492</v>
+        <v>465</v>
       </c>
       <c r="E122" t="s">
-        <v>499</v>
+        <v>471</v>
       </c>
       <c r="F122" t="s">
         <v>392</v>
@@ -8646,10 +8565,10 @@
         <v>80</v>
       </c>
       <c r="C123" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D123" t="s">
-        <v>493</v>
+        <v>466</v>
       </c>
       <c r="F123" t="s">
         <v>392</v>
@@ -8663,10 +8582,10 @@
         <v>80</v>
       </c>
       <c r="C124" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D124" t="s">
-        <v>494</v>
+        <v>467</v>
       </c>
       <c r="F124" t="s">
         <v>392</v>
@@ -8680,10 +8599,10 @@
         <v>80</v>
       </c>
       <c r="C125" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D125" t="s">
-        <v>495</v>
+        <v>468</v>
       </c>
       <c r="F125" t="s">
         <v>392</v>
@@ -8697,7 +8616,7 @@
         <v>80</v>
       </c>
       <c r="C126" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D126" t="s">
         <v>327</v>
@@ -8726,7 +8645,7 @@
         <v>80</v>
       </c>
       <c r="C127" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D127" t="s">
         <v>329</v>
@@ -8755,7 +8674,7 @@
         <v>80</v>
       </c>
       <c r="C128" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D128" t="s">
         <v>331</v>
@@ -8784,7 +8703,7 @@
         <v>80</v>
       </c>
       <c r="C129" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D129" t="s">
         <v>333</v>
@@ -8813,7 +8732,7 @@
         <v>80</v>
       </c>
       <c r="C130" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D130" t="s">
         <v>335</v>
@@ -8842,7 +8761,7 @@
         <v>80</v>
       </c>
       <c r="C131" t="s">
-        <v>489</v>
+        <v>462</v>
       </c>
       <c r="D131" t="s">
         <v>337</v>
@@ -8871,13 +8790,13 @@
         <v>82</v>
       </c>
       <c r="C132" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D132" t="s">
-        <v>500</v>
+        <v>472</v>
       </c>
       <c r="E132" t="s">
-        <v>501</v>
+        <v>473</v>
       </c>
       <c r="F132" t="s">
         <v>392</v>
@@ -8886,10 +8805,10 @@
         <v>393</v>
       </c>
       <c r="H132" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="I132" t="s">
-        <v>504</v>
+        <v>476</v>
       </c>
       <c r="J132" t="s">
         <v>423</v>
@@ -8903,13 +8822,13 @@
         <v>82</v>
       </c>
       <c r="C133" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D133" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="E133" t="s">
-        <v>507</v>
+        <v>478</v>
       </c>
       <c r="F133" t="s">
         <v>392</v>
@@ -8918,10 +8837,10 @@
         <v>393</v>
       </c>
       <c r="H133" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="I133" t="s">
-        <v>506</v>
+        <v>477</v>
       </c>
       <c r="J133" t="s">
         <v>423</v>
@@ -8935,13 +8854,13 @@
         <v>82</v>
       </c>
       <c r="C134" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D134" t="s">
         <v>240</v>
       </c>
       <c r="E134" t="s">
-        <v>512</v>
+        <v>483</v>
       </c>
       <c r="F134" t="s">
         <v>392</v>
@@ -8950,13 +8869,13 @@
         <v>393</v>
       </c>
       <c r="H134" t="s">
-        <v>511</v>
+        <v>482</v>
       </c>
       <c r="I134" t="s">
-        <v>508</v>
+        <v>479</v>
       </c>
       <c r="J134" t="s">
-        <v>532</v>
+        <v>503</v>
       </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.25">
@@ -8967,13 +8886,13 @@
         <v>82</v>
       </c>
       <c r="C135" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D135" t="s">
-        <v>518</v>
+        <v>489</v>
       </c>
       <c r="E135" t="s">
-        <v>513</v>
+        <v>484</v>
       </c>
       <c r="F135" t="s">
         <v>392</v>
@@ -8982,10 +8901,10 @@
         <v>393</v>
       </c>
       <c r="H135" t="s">
-        <v>511</v>
+        <v>482</v>
       </c>
       <c r="I135" t="s">
-        <v>509</v>
+        <v>480</v>
       </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.25">
@@ -8996,13 +8915,13 @@
         <v>82</v>
       </c>
       <c r="C136" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D136" t="s">
         <v>388</v>
       </c>
       <c r="E136" t="s">
-        <v>514</v>
+        <v>485</v>
       </c>
       <c r="F136" t="s">
         <v>392</v>
@@ -9011,13 +8930,13 @@
         <v>393</v>
       </c>
       <c r="H136" t="s">
-        <v>511</v>
+        <v>482</v>
       </c>
       <c r="I136" t="s">
         <v>403</v>
       </c>
       <c r="J136" t="s">
-        <v>532</v>
+        <v>503</v>
       </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.25">
@@ -9028,13 +8947,13 @@
         <v>82</v>
       </c>
       <c r="C137" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D137" t="s">
-        <v>490</v>
+        <v>463</v>
       </c>
       <c r="E137" t="s">
-        <v>515</v>
+        <v>486</v>
       </c>
       <c r="F137" t="s">
         <v>392</v>
@@ -9043,13 +8962,13 @@
         <v>393</v>
       </c>
       <c r="H137" t="s">
-        <v>511</v>
+        <v>482</v>
       </c>
       <c r="I137" t="s">
-        <v>510</v>
+        <v>481</v>
       </c>
       <c r="J137" t="s">
-        <v>532</v>
+        <v>503</v>
       </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.25">
@@ -9060,13 +8979,13 @@
         <v>82</v>
       </c>
       <c r="C138" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D138" t="s">
         <v>442</v>
       </c>
       <c r="E138" t="s">
-        <v>516</v>
+        <v>487</v>
       </c>
       <c r="F138" t="s">
         <v>392</v>
@@ -9075,13 +8994,13 @@
         <v>393</v>
       </c>
       <c r="H138" t="s">
-        <v>511</v>
+        <v>482</v>
       </c>
       <c r="I138" t="s">
         <v>406</v>
       </c>
       <c r="J138" t="s">
-        <v>532</v>
+        <v>503</v>
       </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.25">
@@ -9092,28 +9011,28 @@
         <v>82</v>
       </c>
       <c r="C139" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D139" t="s">
         <v>287</v>
       </c>
       <c r="E139" t="s">
-        <v>519</v>
+        <v>490</v>
       </c>
       <c r="F139" t="s">
-        <v>497</v>
+        <v>470</v>
       </c>
       <c r="G139" t="s">
         <v>393</v>
       </c>
       <c r="H139" t="s">
+        <v>475</v>
+      </c>
+      <c r="I139" t="s">
+        <v>488</v>
+      </c>
+      <c r="J139" t="s">
         <v>503</v>
-      </c>
-      <c r="I139" t="s">
-        <v>517</v>
-      </c>
-      <c r="J139" t="s">
-        <v>532</v>
       </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.25">
@@ -9124,13 +9043,13 @@
         <v>82</v>
       </c>
       <c r="C140" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D140" t="s">
-        <v>528</v>
+        <v>499</v>
       </c>
       <c r="E140" t="s">
-        <v>524</v>
+        <v>495</v>
       </c>
       <c r="F140" t="s">
         <v>392</v>
@@ -9139,10 +9058,10 @@
         <v>393</v>
       </c>
       <c r="H140" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="I140" t="s">
-        <v>520</v>
+        <v>491</v>
       </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.25">
@@ -9153,13 +9072,13 @@
         <v>82</v>
       </c>
       <c r="C141" t="s">
+        <v>469</v>
+      </c>
+      <c r="D141" t="s">
+        <v>500</v>
+      </c>
+      <c r="E141" t="s">
         <v>496</v>
-      </c>
-      <c r="D141" t="s">
-        <v>529</v>
-      </c>
-      <c r="E141" t="s">
-        <v>525</v>
       </c>
       <c r="F141" t="s">
         <v>392</v>
@@ -9168,10 +9087,10 @@
         <v>393</v>
       </c>
       <c r="H141" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="I141" t="s">
-        <v>521</v>
+        <v>492</v>
       </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.25">
@@ -9182,13 +9101,13 @@
         <v>82</v>
       </c>
       <c r="C142" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D142" t="s">
-        <v>530</v>
+        <v>501</v>
       </c>
       <c r="E142" t="s">
-        <v>526</v>
+        <v>497</v>
       </c>
       <c r="F142" t="s">
         <v>392</v>
@@ -9197,10 +9116,10 @@
         <v>393</v>
       </c>
       <c r="H142" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="I142" t="s">
-        <v>522</v>
+        <v>493</v>
       </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.25">
@@ -9211,13 +9130,13 @@
         <v>82</v>
       </c>
       <c r="C143" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D143" t="s">
-        <v>531</v>
+        <v>502</v>
       </c>
       <c r="E143" t="s">
-        <v>527</v>
+        <v>498</v>
       </c>
       <c r="F143" t="s">
         <v>392</v>
@@ -9226,10 +9145,10 @@
         <v>393</v>
       </c>
       <c r="H143" t="s">
-        <v>503</v>
+        <v>475</v>
       </c>
       <c r="I143" t="s">
-        <v>523</v>
+        <v>494</v>
       </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.25">
@@ -9240,7 +9159,7 @@
         <v>82</v>
       </c>
       <c r="C144" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D144" t="s">
         <v>327</v>
@@ -9269,7 +9188,7 @@
         <v>82</v>
       </c>
       <c r="C145" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D145" t="s">
         <v>329</v>
@@ -9298,7 +9217,7 @@
         <v>82</v>
       </c>
       <c r="C146" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D146" t="s">
         <v>331</v>
@@ -9327,7 +9246,7 @@
         <v>82</v>
       </c>
       <c r="C147" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D147" t="s">
         <v>333</v>
@@ -9356,7 +9275,7 @@
         <v>82</v>
       </c>
       <c r="C148" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D148" t="s">
         <v>335</v>
@@ -9385,7 +9304,7 @@
         <v>82</v>
       </c>
       <c r="C149" t="s">
-        <v>496</v>
+        <v>469</v>
       </c>
       <c r="D149" t="s">
         <v>337</v>
@@ -9660,21 +9579,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A1" s="91" t="s">
-        <v>468</v>
-      </c>
+      <c r="A1" s="91"/>
     </row>
     <row r="2" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="A2" s="91" t="s">
-        <v>469</v>
-      </c>
-      <c r="E2" s="92" t="str">
-        <f>SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(G2,FIND("]",G2)),"]",""),"[",""),"    ","")</f>
-        <v>territory_key</v>
-      </c>
-      <c r="G2" s="83" t="s">
-        <v>470</v>
-      </c>
+      <c r="A2" s="91"/>
+      <c r="E2" s="92"/>
       <c r="M2" s="87"/>
       <c r="N2" s="88"/>
       <c r="Q2" s="87"/>
@@ -9684,22 +9593,7 @@
     </row>
     <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" s="84"/>
-      <c r="B3" s="83">
-        <v>1</v>
-      </c>
-      <c r="C3" s="83" t="s">
-        <v>406</v>
-      </c>
-      <c r="D3" s="83" t="s">
-        <v>444</v>
-      </c>
-      <c r="E3" s="92" t="str">
-        <f t="shared" ref="E3:E6" si="0">SUBSTITUTE(SUBSTITUTE(SUBSTITUTE(LEFT(G3,FIND("]",G3)),"]",""),"[",""),"    ","")</f>
-        <v>territory_name_bk</v>
-      </c>
-      <c r="G3" s="83" t="s">
-        <v>459</v>
-      </c>
+      <c r="E3" s="92"/>
       <c r="Q3" s="87"/>
       <c r="R3" s="88"/>
       <c r="S3" s="87"/>
@@ -9709,22 +9603,7 @@
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" s="84"/>
-      <c r="B4" s="83">
-        <v>2</v>
-      </c>
-      <c r="C4" s="83" t="s">
-        <v>429</v>
-      </c>
-      <c r="D4" s="83" t="s">
-        <v>432</v>
-      </c>
-      <c r="E4" s="92" t="str">
-        <f t="shared" si="0"/>
-        <v>territory_group</v>
-      </c>
-      <c r="G4" s="83" t="s">
-        <v>460</v>
-      </c>
+      <c r="E4" s="92"/>
       <c r="Q4" s="87"/>
       <c r="R4" s="88"/>
       <c r="S4" s="87"/>
@@ -9734,22 +9613,9 @@
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" s="84"/>
-      <c r="B5" s="84">
-        <v>3</v>
-      </c>
-      <c r="C5" s="84" t="s">
-        <v>430</v>
-      </c>
-      <c r="D5" s="83" t="s">
-        <v>433</v>
-      </c>
-      <c r="E5" s="92" t="str">
-        <f t="shared" si="0"/>
-        <v>country_region_code</v>
-      </c>
-      <c r="G5" s="83" t="s">
-        <v>461</v>
-      </c>
+      <c r="B5" s="84"/>
+      <c r="C5" s="84"/>
+      <c r="E5" s="92"/>
       <c r="Q5" s="87"/>
       <c r="R5" s="88"/>
       <c r="S5" s="87"/>
@@ -9759,159 +9625,49 @@
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" s="84"/>
-      <c r="B6" s="83">
-        <v>4</v>
-      </c>
-      <c r="C6" s="83" t="s">
-        <v>431</v>
-      </c>
-      <c r="D6" s="83" t="s">
-        <v>434</v>
-      </c>
-      <c r="E6" s="92" t="str">
-        <f t="shared" si="0"/>
-        <v>country_name</v>
-      </c>
-      <c r="G6" s="83" t="s">
-        <v>462</v>
-      </c>
+      <c r="E6" s="92"/>
       <c r="Q6" s="87"/>
       <c r="R6" s="88"/>
       <c r="Y6" s="87"/>
     </row>
     <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" s="84"/>
-      <c r="B7" s="83">
-        <v>5</v>
-      </c>
-      <c r="C7" s="83" t="s">
-        <v>445</v>
-      </c>
-      <c r="D7" s="83" t="s">
-        <v>446</v>
-      </c>
-      <c r="G7" s="83" t="s">
-        <v>457</v>
-      </c>
       <c r="Q7" s="87"/>
       <c r="R7" s="88"/>
       <c r="Y7" s="87"/>
     </row>
     <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" s="84"/>
-      <c r="B8" s="83">
-        <v>6</v>
-      </c>
-      <c r="C8" s="83" t="s">
-        <v>447</v>
-      </c>
-      <c r="D8" s="83" t="s">
-        <v>448</v>
-      </c>
-      <c r="E8" s="83" t="str">
-        <f t="shared" ref="E8:E12" si="1">LEFT(G8, FIND("]", G8))</f>
-        <v>    [sys_insert_date]</v>
-      </c>
-      <c r="G8" s="83" t="s">
-        <v>463</v>
-      </c>
       <c r="Q8" s="87"/>
       <c r="R8" s="88"/>
       <c r="Y8" s="87"/>
     </row>
     <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" s="84"/>
-      <c r="B9" s="83">
-        <v>7</v>
-      </c>
-      <c r="C9" s="83" t="s">
-        <v>449</v>
-      </c>
-      <c r="D9" s="83" t="s">
-        <v>450</v>
-      </c>
-      <c r="E9" s="83" t="str">
-        <f t="shared" si="1"/>
-        <v>    [sys_update_date]</v>
-      </c>
-      <c r="G9" s="83" t="s">
-        <v>464</v>
-      </c>
       <c r="N9" s="87"/>
       <c r="O9" s="88"/>
       <c r="V9" s="87"/>
     </row>
     <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" s="84"/>
-      <c r="B10" s="83">
-        <v>8</v>
-      </c>
-      <c r="C10" s="83" t="s">
-        <v>451</v>
-      </c>
-      <c r="D10" s="83" t="s">
-        <v>452</v>
-      </c>
-      <c r="E10" s="83" t="str">
-        <f t="shared" si="1"/>
-        <v>    [sys_delete_date]</v>
-      </c>
-      <c r="G10" s="83" t="s">
-        <v>465</v>
-      </c>
       <c r="N10" s="87"/>
       <c r="O10" s="88"/>
       <c r="V10" s="87"/>
     </row>
     <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" s="84"/>
-      <c r="B11" s="83">
-        <v>9</v>
-      </c>
-      <c r="C11" s="83" t="s">
-        <v>453</v>
-      </c>
-      <c r="D11" s="83" t="s">
-        <v>454</v>
-      </c>
-      <c r="E11" s="83" t="str">
-        <f t="shared" si="1"/>
-        <v>    [sys_hash_value]</v>
-      </c>
-      <c r="G11" s="83" t="s">
-        <v>466</v>
-      </c>
       <c r="N11" s="87"/>
       <c r="O11" s="88"/>
       <c r="V11" s="87"/>
     </row>
     <row r="12" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A12" s="84"/>
-      <c r="B12" s="83">
-        <v>10</v>
-      </c>
-      <c r="C12" s="83" t="s">
-        <v>455</v>
-      </c>
-      <c r="D12" s="83" t="s">
-        <v>456</v>
-      </c>
-      <c r="E12" s="83" t="str">
-        <f t="shared" si="1"/>
-        <v>    [sys_data_source]</v>
-      </c>
-      <c r="G12" s="83" t="s">
-        <v>467</v>
-      </c>
       <c r="N12" s="87"/>
       <c r="O12" s="88"/>
       <c r="V12" s="87"/>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A13" s="84"/>
-      <c r="G13" s="83" t="s">
-        <v>458</v>
-      </c>
       <c r="N13" s="87"/>
       <c r="O13" s="88"/>
       <c r="V13" s="87"/>

</xml_diff>